<commit_message>
Herstarten LLL, na computer crash en het afwerken van eindwerken
in februari is oude laptop gecrasht waardoor ik mijn geschiedenis van Python deels kwijt ben.
Door het volgen van C# geraakte ik wat in de war door het verschil in coderen.
daarom besloten om LLL even on hold te zetten.
ga vlug per dag 4 lessen herbekijken om terug mee te zijn met de syntax van Python
</commit_message>
<xml_diff>
--- a/Opstart_documenten/Actieplan_Python.xlsx
+++ b/Opstart_documenten/Actieplan_Python.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f020cdb928d38096/Programmeren/Odisee/LevensLang_Leren/LLL-BartBrondeel-2526/Opstart_documenten/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FE0E0FB-1E8E-46C2-9B64-4F2896E6678C}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF222FDC-71DC-407D-B41D-183807DF28F0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Actieplan" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
   <si>
     <t>Nr</t>
   </si>
@@ -163,6 +163,12 @@
   </si>
   <si>
     <t>Geschatte duur (uren)</t>
+  </si>
+  <si>
+    <t>er is rekening gehouden met de krokus en paasvakantie</t>
+  </si>
+  <si>
+    <t>+ 2 weken om zolder om te bouwen naar studeer ruimte</t>
   </si>
 </sst>
 </file>
@@ -294,7 +300,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -332,6 +338,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -347,10 +354,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -640,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -746,7 +749,7 @@
         <v>45945</v>
       </c>
       <c r="E4" s="11">
-        <v>45987</v>
+        <v>46010</v>
       </c>
       <c r="F4" s="10">
         <v>45</v>
@@ -772,10 +775,10 @@
         <v>18</v>
       </c>
       <c r="D5" s="11">
-        <v>45988</v>
+        <v>46027</v>
       </c>
       <c r="E5" s="11">
-        <v>46029</v>
+        <v>46087</v>
       </c>
       <c r="F5" s="10">
         <v>27</v>
@@ -801,10 +804,10 @@
         <v>19</v>
       </c>
       <c r="D6" s="11">
-        <v>46030</v>
+        <v>46090</v>
       </c>
       <c r="E6" s="11">
-        <v>46071</v>
+        <v>46150</v>
       </c>
       <c r="F6" s="10">
         <v>50</v>
@@ -857,10 +860,10 @@
         <v>17</v>
       </c>
       <c r="D9" s="12">
-        <v>46071</v>
+        <v>46132</v>
       </c>
       <c r="E9" s="12">
-        <v>46105</v>
+        <v>46166</v>
       </c>
       <c r="F9" s="2">
         <f>SUM(F10:F15)</f>
@@ -884,10 +887,10 @@
         <v>18</v>
       </c>
       <c r="D10" s="11">
-        <v>46071</v>
+        <v>46132</v>
       </c>
       <c r="E10" s="11">
-        <v>46087</v>
+        <v>46136</v>
       </c>
       <c r="F10" s="10">
         <v>12</v>
@@ -910,10 +913,10 @@
         <v>18</v>
       </c>
       <c r="D11" s="11">
-        <v>46090</v>
+        <v>46139</v>
       </c>
       <c r="E11" s="11">
-        <v>46105</v>
+        <v>46143</v>
       </c>
       <c r="F11" s="10">
         <v>12</v>
@@ -936,10 +939,10 @@
         <v>19</v>
       </c>
       <c r="D12" s="11">
-        <v>46111</v>
+        <v>46146</v>
       </c>
       <c r="E12" s="11">
-        <v>46113</v>
+        <v>46146</v>
       </c>
       <c r="F12" s="10">
         <v>4</v>
@@ -959,8 +962,12 @@
       <c r="C13" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
+      <c r="D13" s="11">
+        <v>46147</v>
+      </c>
+      <c r="E13" s="11">
+        <v>46150</v>
+      </c>
       <c r="F13" s="10">
         <v>12</v>
       </c>
@@ -1007,7 +1014,7 @@
         <v>17</v>
       </c>
       <c r="D16" s="12">
-        <v>46119</v>
+        <v>46153</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>20</v>
@@ -1034,10 +1041,10 @@
         <v>18</v>
       </c>
       <c r="D17" s="11">
-        <v>46119</v>
+        <v>46153</v>
       </c>
       <c r="E17" s="11">
-        <v>46139</v>
+        <v>46161</v>
       </c>
       <c r="F17" s="10">
         <v>15</v>
@@ -1060,10 +1067,10 @@
         <v>18</v>
       </c>
       <c r="D18" s="11">
-        <v>46140</v>
+        <v>46162</v>
       </c>
       <c r="E18" s="11">
-        <v>46164</v>
+        <v>46169</v>
       </c>
       <c r="F18" s="10">
         <v>15</v>
@@ -1086,10 +1093,10 @@
         <v>19</v>
       </c>
       <c r="D19" s="11">
-        <v>46167</v>
+        <v>46170</v>
       </c>
       <c r="E19" s="11">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="F19" s="10">
         <v>10</v>
@@ -1142,6 +1149,16 @@
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
         <v>101.25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="19" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update actieplan, logbook en log 26W17
</commit_message>
<xml_diff>
--- a/Opstart_documenten/Actieplan_Python.xlsx
+++ b/Opstart_documenten/Actieplan_Python.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\Odisee\LLL-BartBrondeel-2526\Opstart_documenten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E4C0028-3BDC-4D66-85FD-02D406499F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB1AE63-C8DD-410D-9210-385ED3C00685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="60" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="60" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Actieplan" sheetId="1" r:id="rId1"/>
@@ -787,7 +787,7 @@
       <c r="H5" s="10"/>
       <c r="I5" s="10">
         <f>('Werkelijke uren'!D62)</f>
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>22</v>
@@ -833,7 +833,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>115.25</v>
+        <v>121.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>115.25</v>
+        <v>121.25</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -1536,16 +1536,25 @@
       <c r="B46">
         <v>44</v>
       </c>
+      <c r="C46">
+        <v>2</v>
+      </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
         <v>45</v>
       </c>
+      <c r="C47">
+        <v>2</v>
+      </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
         <v>46</v>
       </c>
+      <c r="C48">
+        <v>2</v>
+      </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49">
@@ -1618,7 +1627,7 @@
       </c>
       <c r="D62">
         <f>SUM(C33:C62)</f>
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.25">
@@ -1831,7 +1840,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>115.25</v>
+        <v>121.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Actieplan en Logbook
</commit_message>
<xml_diff>
--- a/Opstart_documenten/Actieplan_Python.xlsx
+++ b/Opstart_documenten/Actieplan_Python.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\Odisee\LLL-BartBrondeel-2526\Opstart_documenten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67280757-51D0-4D8F-923B-4144D6FE4454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550814C3-C405-4B3F-9F97-D461B1773B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="60" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -826,7 +826,7 @@
       <c r="H6" s="10"/>
       <c r="I6" s="10">
         <f>('Werkelijke uren'!D102)</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J6" s="10" t="s">
         <v>23</v>
@@ -843,7 +843,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>153.25</v>
+        <v>161.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>153.25</v>
+        <v>161.25</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -1718,21 +1718,33 @@
       <c r="B67">
         <v>65</v>
       </c>
+      <c r="C67">
+        <v>2</v>
+      </c>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68">
         <v>66</v>
       </c>
+      <c r="C68">
+        <v>2</v>
+      </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69">
         <v>67</v>
       </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70">
         <v>68</v>
       </c>
+      <c r="C70">
+        <v>2</v>
+      </c>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71">
@@ -1895,7 +1907,7 @@
       </c>
       <c r="D102">
         <f>SUM(C63:C102)</f>
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.25">
@@ -1904,7 +1916,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>153.25</v>
+        <v>161.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Actieplan en Logbook 26W19 toegevoegd
</commit_message>
<xml_diff>
--- a/Opstart_documenten/Actieplan_Python.xlsx
+++ b/Opstart_documenten/Actieplan_Python.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\Odisee\LLL-BartBrondeel-2526\Opstart_documenten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550814C3-C405-4B3F-9F97-D461B1773B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ACBD4AF-328D-4B09-BDEC-71E8D8A3AD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="60" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -826,7 +826,7 @@
       <c r="H6" s="10"/>
       <c r="I6" s="10">
         <f>('Werkelijke uren'!D102)</f>
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J6" s="10" t="s">
         <v>23</v>
@@ -843,7 +843,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>161.25</v>
+        <v>169.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -907,7 +907,9 @@
       </c>
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
+      <c r="I10" s="10">
+        <v>4</v>
+      </c>
       <c r="J10" s="10" t="s">
         <v>24</v>
       </c>
@@ -997,7 +999,7 @@
       <c r="H14" s="10"/>
       <c r="I14" s="10">
         <f>SUM(I10:I13)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J14" s="10"/>
     </row>
@@ -1158,7 +1160,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>161.25</v>
+        <v>173.25</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -1750,21 +1752,33 @@
       <c r="B71">
         <v>69</v>
       </c>
+      <c r="C71">
+        <v>2</v>
+      </c>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72">
         <v>70</v>
       </c>
+      <c r="C72">
+        <v>2</v>
+      </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73">
         <v>71</v>
       </c>
+      <c r="C73">
+        <v>2</v>
+      </c>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74">
         <v>72</v>
       </c>
+      <c r="C74">
+        <v>2</v>
+      </c>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75">
@@ -1907,7 +1921,7 @@
       </c>
       <c r="D102">
         <f>SUM(C63:C102)</f>
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.25">
@@ -1916,7 +1930,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>161.25</v>
+        <v>169.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>